<commit_message>
subiendo version 0.3.0 - acceso a estudiantes : feature/student
</commit_message>
<xml_diff>
--- a/docs/scrum_artifacts/product_backlog.xlsx
+++ b/docs/scrum_artifacts/product_backlog.xlsx
@@ -5,16 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MIGUEL ÁNGEL\Documents\Universidad de Nariño\Semestres\Quinto semestre\Ingenieria de software III\CambridgeAcademy\docs-ver2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MIGUEL ÁNGEL\Documents\Universidad de Nariño\Semestres\Quinto semestre\Ingenieria de software III\CambridgeAcademy\new_ver\sprint3\ca_v0.3.0\docs\scrum_artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CF187B5-4130-4206-AF7A-248027BF4616}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E2E6C4-B85B-4AB8-B4B1-308CD051D199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$G$31</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -25,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
   <si>
     <t>ID</t>
   </si>
@@ -316,9 +319,6 @@
   </si>
   <si>
     <t>Control académico administrativo</t>
-  </si>
-  <si>
-    <t>Por terminar.</t>
   </si>
 </sst>
 </file>
@@ -654,6 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.7109375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -683,7 +684,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
@@ -706,7 +707,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -726,10 +727,10 @@
         <v>1</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -749,10 +750,10 @@
         <v>1</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -772,10 +773,10 @@
         <v>1</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -795,10 +796,10 @@
         <v>1</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -818,10 +819,10 @@
         <v>1</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -841,10 +842,10 @@
         <v>1</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>42</v>
       </c>
@@ -864,10 +865,10 @@
         <v>2</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -887,10 +888,10 @@
         <v>2</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
@@ -910,10 +911,10 @@
         <v>2</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -933,10 +934,10 @@
         <v>2</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -956,10 +957,10 @@
         <v>2</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -979,10 +980,10 @@
         <v>2</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1002,10 +1003,10 @@
         <v>2</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
@@ -1025,10 +1026,10 @@
         <v>2</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -1048,7 +1049,7 @@
         <v>2</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1071,7 +1072,7 @@
         <v>3</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1094,7 +1095,7 @@
         <v>3</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1117,7 +1118,7 @@
         <v>3</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1140,7 +1141,7 @@
         <v>3</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1163,7 +1164,7 @@
         <v>3</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1186,7 +1187,7 @@
         <v>3</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1209,10 +1210,10 @@
         <v>3</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>77</v>
       </c>
@@ -1235,7 +1236,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>80</v>
       </c>
@@ -1258,7 +1259,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>83</v>
       </c>
@@ -1281,7 +1282,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>86</v>
       </c>
@@ -1304,7 +1305,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>89</v>
       </c>
@@ -1327,7 +1328,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>92</v>
       </c>
@@ -1350,7 +1351,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>94</v>
       </c>
@@ -1374,6 +1375,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G31" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="5">
+      <filters>
+        <filter val="3"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
subiendo version 0.4.0 - profesores y notas : feature/professor
</commit_message>
<xml_diff>
--- a/docs/scrum_artifacts/product_backlog.xlsx
+++ b/docs/scrum_artifacts/product_backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MIGUEL ÁNGEL\Documents\Universidad de Nariño\Semestres\Quinto semestre\Ingenieria de software III\CambridgeAcademy\new_ver\sprint3\ca_v0.3.0\docs\scrum_artifacts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MIGUEL ÁNGEL\Documents\Universidad de Nariño\Semestres\Quinto semestre\Ingenieria de software III\CambridgeAcademy\new_ver\sprint4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86E2E6C4-B85B-4AB8-B4B1-308CD051D199}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AEDFDA-9F9E-4892-B924-E335923DBE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1052,7 +1052,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>56</v>
       </c>
@@ -1075,7 +1075,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>59</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>62</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>65</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>68</v>
       </c>
@@ -1167,7 +1167,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>71</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>74</v>
       </c>
@@ -1213,7 +1213,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>77</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>80</v>
       </c>
@@ -1259,7 +1259,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>83</v>
       </c>
@@ -1282,7 +1282,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>86</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>89</v>
       </c>
@@ -1328,7 +1328,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>92</v>
       </c>
@@ -1351,7 +1351,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>94</v>
       </c>
@@ -1378,7 +1378,7 @@
   <autoFilter ref="A1:G31" xr:uid="{00000000-0001-0000-0000-000000000000}">
     <filterColumn colId="5">
       <filters>
-        <filter val="3"/>
+        <filter val="4"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Subiendo version 1.0.0 - CA Funcional ; Artefactos scrum completado
</commit_message>
<xml_diff>
--- a/docs/scrum_artifacts/product_backlog.xlsx
+++ b/docs/scrum_artifacts/product_backlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MIGUEL ÁNGEL\Documents\Universidad de Nariño\Semestres\Quinto semestre\Ingenieria de software III\CambridgeAcademy\new_ver\sprint4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MIGUEL ÁNGEL\Documents\Universidad de Nariño\Semestres\Quinto semestre\Ingenieria de software III\CambridgeAcademy\new_ver\sprint4\ca_v0.4.0\docs\scrum_artifacts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19AEDFDA-9F9E-4892-B924-E335923DBE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7904F622-FEB2-47F0-A4B4-1296418BB46E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="10455" windowHeight="10905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="96">
   <si>
     <t>ID</t>
   </si>
@@ -163,9 +163,6 @@
   </si>
   <si>
     <t>Mantener información actualizada</t>
-  </si>
-  <si>
-    <t>Por iniciar</t>
   </si>
   <si>
     <t>Eliminar datos de estudiantes</t>
@@ -654,7 +651,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.7109375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -684,7 +680,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
@@ -707,7 +703,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -730,7 +726,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -753,7 +749,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -776,7 +772,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -799,7 +795,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -822,7 +818,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
@@ -845,7 +841,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>42</v>
       </c>
@@ -868,7 +864,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -876,10 +872,10 @@
         <v>15</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>26</v>
@@ -891,7 +887,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
@@ -899,10 +895,10 @@
         <v>15</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>26</v>
@@ -914,7 +910,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -922,7 +918,7 @@
         <v>15</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>44</v>
@@ -937,7 +933,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -945,10 +941,10 @@
         <v>15</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>26</v>
@@ -960,7 +956,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -968,10 +964,10 @@
         <v>15</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>29</v>
@@ -983,7 +979,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -991,7 +987,7 @@
         <v>15</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>44</v>
@@ -1006,7 +1002,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
@@ -1014,10 +1010,10 @@
         <v>15</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>26</v>
@@ -1029,7 +1025,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -1037,10 +1033,10 @@
         <v>15</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>29</v>
@@ -1052,18 +1048,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>58</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>26</v>
@@ -1075,18 +1071,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>26</v>
@@ -1098,18 +1094,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C20" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>64</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>29</v>
@@ -1121,18 +1117,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>26</v>
@@ -1144,18 +1140,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D22" s="1" t="s">
         <v>69</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>29</v>
@@ -1167,18 +1163,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C23" s="1" t="s">
+      <c r="D23" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>29</v>
@@ -1190,18 +1186,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>76</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>26</v>
@@ -1215,16 +1211,16 @@
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C25" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>26</v>
@@ -1233,21 +1229,21 @@
         <v>4</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C26" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="D26" s="1" t="s">
-        <v>82</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>26</v>
@@ -1256,21 +1252,21 @@
         <v>4</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>26</v>
@@ -1279,21 +1275,21 @@
         <v>4</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>88</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>29</v>
@@ -1302,21 +1298,21 @@
         <v>4</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C29" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D29" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>29</v>
@@ -1325,21 +1321,21 @@
         <v>4</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>29</v>
@@ -1348,21 +1344,21 @@
         <v>4</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C31" s="1" t="s">
+      <c r="D31" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>30</v>
@@ -1371,17 +1367,11 @@
         <v>4</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G31" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="4"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:G31" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>